<commit_message>
feat: serverseitige Benachrichtigungs-Mails (Resend) an beide + Portal-Hinweis
Auf Wunsch reaktiviert: bei neuer Nachricht/Anfrage bekommt die andere Seite
(Provider bzw. Eigner) eine Resend-Mail mit Hinweis, im Portal zu antworten.
- notify-message: Portal-Hinweis in Text + HTML ergänzt
- Aufrufe wieder eingebunden: Owner-Chat, Provider-Chat, Erst-Anfrage

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Skipily_Business_Model.xlsx
+++ b/Skipily_Business_Model.xlsx
@@ -1,25 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ekkehart/Documents/01-Projekte/Programmieren/BoatCare/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{869C43D5-F50A-7845-BFDE-720FE2627200}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB79B030-85E2-FC46-A32C-57B73ACDA679}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10000" yWindow="7380" windowWidth="31760" windowHeight="17760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="30240" windowHeight="17760" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1_Annahmen" sheetId="1" r:id="rId1"/>
     <sheet name="2_Pricing" sheetId="2" r:id="rId2"/>
     <sheet name="3_Investment" sheetId="3" r:id="rId3"/>
     <sheet name="4_Kosten" sheetId="4" r:id="rId4"/>
-    <sheet name="5_Umsatz_Prognose" sheetId="5" r:id="rId5"/>
-    <sheet name="6_GuV_Breakeven" sheetId="6" r:id="rId6"/>
-    <sheet name="7_Verlauf_Charts" sheetId="7" r:id="rId7"/>
+    <sheet name="5_Umsatz_Prognose (2)" sheetId="10" r:id="rId5"/>
+    <sheet name="5_Umsatz_Prognose" sheetId="5" r:id="rId6"/>
+    <sheet name="6_GuV_Breakeven" sheetId="6" r:id="rId7"/>
+    <sheet name="7_Verlauf_Charts" sheetId="7" r:id="rId8"/>
+    <sheet name="8_Bewertung" sheetId="8" r:id="rId9"/>
+    <sheet name="9_Beteiligung" sheetId="9" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +42,100 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="258">
+  <si>
+    <t>PRICING-STRATEGIE: Privat-User &amp; Service-Provider</t>
+  </si>
+  <si>
+    <t>Privat-User (B2C, Freemium)</t>
+  </si>
+  <si>
+    <t>Tier</t>
+  </si>
+  <si>
+    <t>Preis/Monat</t>
+  </si>
+  <si>
+    <t>Preis/Jahr</t>
+  </si>
+  <si>
+    <t>Ø Blended €/Mon</t>
+  </si>
+  <si>
+    <t>Zielgruppe</t>
+  </si>
+  <si>
+    <t>Free</t>
+  </si>
+  <si>
+    <t>Einsteiger / Lead-Gen</t>
+  </si>
+  <si>
+    <t>Skipily Plus</t>
+  </si>
+  <si>
+    <t>Hobby-Skipper, 1-2 Boote</t>
+  </si>
+  <si>
+    <t>Skipily Pro</t>
+  </si>
+  <si>
+    <t>Eigner-Profis, Mehrboot, Charterer</t>
+  </si>
+  <si>
+    <t>Service-Provider (B2B SaaS + Provisionen)</t>
+  </si>
+  <si>
+    <t>Inhalte</t>
+  </si>
+  <si>
+    <t>Basic Listing</t>
+  </si>
+  <si>
+    <t>Verifiziertes Profil, Map-Pin (Lead-Gen)</t>
+  </si>
+  <si>
+    <t>Provider Starter</t>
+  </si>
+  <si>
+    <t>Foto-Galerie, 5 Promos/Mon, Reviews</t>
+  </si>
+  <si>
+    <t>Provider Pro</t>
+  </si>
+  <si>
+    <t>Unlimited Promos, Shop, Analytics, Top-Placement</t>
+  </si>
+  <si>
+    <t>Provider Enterprise</t>
+  </si>
+  <si>
+    <t>Multi-Location, API, White-Label-Widget</t>
+  </si>
+  <si>
+    <t>Mix-Annahmen (für Umsatzprognose – änderbar)</t>
+  </si>
+  <si>
+    <t>Anteil zahlende Privat → Plus</t>
+  </si>
+  <si>
+    <t>Anteil zahlende Privat → Pro</t>
+  </si>
+  <si>
+    <t>Anteil Provider → Starter</t>
+  </si>
+  <si>
+    <t>Anteil Provider → Pro</t>
+  </si>
+  <si>
+    <t>Anteil Provider → Enterprise</t>
+  </si>
+  <si>
+    <t>ARPU/Monat zahlender Privat-User</t>
+  </si>
+  <si>
+    <t>ARPU/Monat zahlender Provider</t>
+  </si>
   <si>
     <t>SKIPILY – Marktannahmen &amp; Modellparameter (gelbe Zellen = Inputs)</t>
   </si>
@@ -173,99 +269,6 @@
     <t>HINWEIS: Alle gelben Zellen sind Annahmen – einfach ändern, das gesamte Modell rechnet automatisch nach.</t>
   </si>
   <si>
-    <t>PRICING-STRATEGIE: Privat-User &amp; Service-Provider</t>
-  </si>
-  <si>
-    <t>Privat-User (B2C, Freemium)</t>
-  </si>
-  <si>
-    <t>Tier</t>
-  </si>
-  <si>
-    <t>Preis/Monat</t>
-  </si>
-  <si>
-    <t>Preis/Jahr</t>
-  </si>
-  <si>
-    <t>Ø Blended €/Mon</t>
-  </si>
-  <si>
-    <t>Zielgruppe</t>
-  </si>
-  <si>
-    <t>Free</t>
-  </si>
-  <si>
-    <t>Einsteiger / Lead-Gen</t>
-  </si>
-  <si>
-    <t>Skipily Plus</t>
-  </si>
-  <si>
-    <t>Hobby-Skipper, 1-2 Boote</t>
-  </si>
-  <si>
-    <t>Skipily Pro</t>
-  </si>
-  <si>
-    <t>Eigner-Profis, Mehrboot, Charterer</t>
-  </si>
-  <si>
-    <t>Service-Provider (B2B SaaS + Provisionen)</t>
-  </si>
-  <si>
-    <t>Inhalte</t>
-  </si>
-  <si>
-    <t>Basic Listing</t>
-  </si>
-  <si>
-    <t>Verifiziertes Profil, Map-Pin (Lead-Gen)</t>
-  </si>
-  <si>
-    <t>Provider Starter</t>
-  </si>
-  <si>
-    <t>Foto-Galerie, 5 Promos/Mon, Reviews</t>
-  </si>
-  <si>
-    <t>Provider Pro</t>
-  </si>
-  <si>
-    <t>Unlimited Promos, Shop, Analytics, Top-Placement</t>
-  </si>
-  <si>
-    <t>Provider Enterprise</t>
-  </si>
-  <si>
-    <t>Multi-Location, API, White-Label-Widget</t>
-  </si>
-  <si>
-    <t>Mix-Annahmen (für Umsatzprognose – änderbar)</t>
-  </si>
-  <si>
-    <t>Anteil zahlende Privat → Plus</t>
-  </si>
-  <si>
-    <t>Anteil zahlende Privat → Pro</t>
-  </si>
-  <si>
-    <t>Anteil Provider → Starter</t>
-  </si>
-  <si>
-    <t>Anteil Provider → Pro</t>
-  </si>
-  <si>
-    <t>Anteil Provider → Enterprise</t>
-  </si>
-  <si>
-    <t>ARPU/Monat zahlender Privat-User</t>
-  </si>
-  <si>
-    <t>ARPU/Monat zahlender Provider</t>
-  </si>
-  <si>
     <t>INVESTMENT-PLAN (Kapitalbedarf Seed → Series A)</t>
   </si>
   <si>
@@ -395,7 +398,7 @@
     <t>Büro, Co-Working</t>
   </si>
   <si>
-    <t>Software-Tools (Linear, Notion, GitHub Ent., Figma)</t>
+    <t>Software-Tools (Supabase, Google-API,GitHub Ent., Claude)</t>
   </si>
   <si>
     <t>Legal, Buchhaltung, Steuerberatung</t>
@@ -597,18 +600,238 @@
   </si>
   <si>
     <t>Breakeven-Umsatz</t>
+  </si>
+  <si>
+    <t>SKIPILY – Unternehmensbewertung (VC-Methode + Multiples)</t>
+  </si>
+  <si>
+    <t>Verknüpft mit Tab 5 (Umsatz) &amp; Tab 6 (EBITDA). Gelb = Inputs, grün = Querverweis.</t>
+  </si>
+  <si>
+    <t>INPUT-ANNAHMEN (änderbar)</t>
+  </si>
+  <si>
+    <t>Exit-Multiple auf Umsatz (J5)</t>
+  </si>
+  <si>
+    <t>Marktplatz/SaaS 3–6x; konservativ 4x</t>
+  </si>
+  <si>
+    <t>Exit-Multiple auf EBITDA (J5)</t>
+  </si>
+  <si>
+    <t>Profit. SaaS 10–18x</t>
+  </si>
+  <si>
+    <t>Gewichtung Umsatz-Methode</t>
+  </si>
+  <si>
+    <t>Rest = EBITDA-Methode</t>
+  </si>
+  <si>
+    <t>Ziel-IRR Investor (Seed-Risiko)</t>
+  </si>
+  <si>
+    <t>früh: 40–60%</t>
+  </si>
+  <si>
+    <t>Jahre bis Exit</t>
+  </si>
+  <si>
+    <t>Ende Planungshorizont</t>
+  </si>
+  <si>
+    <t>Verwässerung bis Exit (Folgerunden)</t>
+  </si>
+  <si>
+    <t>Seed+Series A; Rest bleibt heutigen Anteilen</t>
+  </si>
+  <si>
+    <t>KENNZAHLEN JAHR 5 (aus Modell)</t>
+  </si>
+  <si>
+    <t>Umsatz Jahr 5 (€)</t>
+  </si>
+  <si>
+    <t>EBITDA Jahr 5 (€)</t>
+  </si>
+  <si>
+    <t>EXIT-WERT (Jahr 5)</t>
+  </si>
+  <si>
+    <t>Exit-Wert auf Umsatz-Basis (€)</t>
+  </si>
+  <si>
+    <t>Exit-Wert auf EBITDA-Basis (€)</t>
+  </si>
+  <si>
+    <t>Exit-Wert gewichtet (€)</t>
+  </si>
+  <si>
+    <t>VC-METHODE – Wert HEUTE</t>
+  </si>
+  <si>
+    <t>Diskontfaktor (1+IRR)^Jahre</t>
+  </si>
+  <si>
+    <t>Unternehmenswert heute – 100% (€)</t>
+  </si>
+  <si>
+    <t>Wert heutiger Anteile nach Verwässerung (€)</t>
+  </si>
+  <si>
+    <t>SENSITIVITÄT – Unternehmenswert heute (100%, €)</t>
+  </si>
+  <si>
+    <t>IRR ↓ / Exit-Umsatz-Multiple →</t>
+  </si>
+  <si>
+    <t>METHODENVERGLEICH → STARTWERT (pre-launch)</t>
+  </si>
+  <si>
+    <t>Methode</t>
+  </si>
+  <si>
+    <t>von (€)</t>
+  </si>
+  <si>
+    <t>bis (€)</t>
+  </si>
+  <si>
+    <t>Substanzwert (Reproduktion Produkt)</t>
+  </si>
+  <si>
+    <t>Quelle: Modell J1 Produkt+Design ~265k</t>
+  </si>
+  <si>
+    <t>Berkus / Scorecard (pre-launch)</t>
+  </si>
+  <si>
+    <t>fertiges Produkt senkt Tech-Risiko</t>
+  </si>
+  <si>
+    <t>DE-Pre-Seed Marktvergleich</t>
+  </si>
+  <si>
+    <t>fertiges Produkt, kein Umsatz</t>
+  </si>
+  <si>
+    <t>VC-Methode (heute, 100%)</t>
+  </si>
+  <si>
+    <t>±20% um VC-Wert oben</t>
+  </si>
+  <si>
+    <t>EMPFOHLENER STARTWERT (Pre-Money)</t>
+  </si>
+  <si>
+    <t>Synthese: oberes Drittel DE-Pre-Seed wg. fertigem Produkt</t>
+  </si>
+  <si>
+    <t>WERTKURVE BEI ZIELERREICHUNG</t>
+  </si>
+  <si>
+    <t>Meilenstein</t>
+  </si>
+  <si>
+    <t>Pre-Money von</t>
+  </si>
+  <si>
+    <t>bis</t>
+  </si>
+  <si>
+    <t>Heute (fertiges Produkt, pre-launch)</t>
+  </si>
+  <si>
+    <t>Ende J1 – Seed (erste zahlende Kunden)</t>
+  </si>
+  <si>
+    <t>J3 – Series A (1,85M Umsatz)</t>
+  </si>
+  <si>
+    <t>J5 – Exit-Fenster (8,68M Umsatz, 38% EBITDA)</t>
+  </si>
+  <si>
+    <t>HINWEIS: Bewertung ist keine Garantie. Werte hängen an den (gelben) Annahmen und an</t>
+  </si>
+  <si>
+    <t>tatsächlicher Traction. Pre-launch zahlt ein Investor den Startwert, nicht den VC-Methoden-Wert.</t>
+  </si>
+  <si>
+    <t>SKIPILY – Beteiligungsrechner (was kostet ein Anteil?)</t>
+  </si>
+  <si>
+    <t>Investment = Pre-Money × Anteil ÷ (1−Anteil) · Post-Money = Pre-Money + Investment</t>
+  </si>
+  <si>
+    <t>Angesetzte Pre-Money-Bewertung (€)</t>
+  </si>
+  <si>
+    <t>Mittelwert Startwert aus Tab 8 (1,2–1,8M) — änderbar</t>
+  </si>
+  <si>
+    <t>A) Was kostet welcher Anteil?</t>
+  </si>
+  <si>
+    <t>Anteil für Investor</t>
+  </si>
+  <si>
+    <t>Investment (€)</t>
+  </si>
+  <si>
+    <t>Post-Money (€)</t>
+  </si>
+  <si>
+    <t>Gründer danach</t>
+  </si>
+  <si>
+    <t>B) Was bekommt der Investor für X €?</t>
+  </si>
+  <si>
+    <t>Anteil %</t>
+  </si>
+  <si>
+    <t>REALITÄTS-CHECK: geplante Seed-Runde</t>
+  </si>
+  <si>
+    <t>Seed-Volumen aus Tab 3 (€)</t>
+  </si>
+  <si>
+    <t>Quelle: Tab 3, Seed Round Q4 J1</t>
+  </si>
+  <si>
+    <t>→ Anteil bei dieser Pre-Money</t>
+  </si>
+  <si>
+    <t>→ Post-Money</t>
+  </si>
+  <si>
+    <t>FAUSTREGEL: Seed-Investoren wollen 10–25%. Mehr als ~25–30% Abgabe</t>
+  </si>
+  <si>
+    <t>in einer frühen Runde schreckt spätere Investoren ab (zu wenig Gründer-Anteil).</t>
+  </si>
+  <si>
+    <t>Lösung bei zu hoher Verwässerung: weniger raisen ODER höhere Pre-Money verhandeln.</t>
+  </si>
+  <si>
+    <t>UMSATZPROGNOSE 2 JAHRE</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="#,##0;\(#,##0\);\-"/>
     <numFmt numFmtId="165" formatCode="0.0%;\(0.0%\);\-"/>
     <numFmt numFmtId="166" formatCode="&quot;€&quot;#,##0;\(&quot;€&quot;#,##0\);\-"/>
+    <numFmt numFmtId="167" formatCode="&quot;€&quot;#,##0.00;\(&quot;€&quot;#,##0.00\);\-"/>
+    <numFmt numFmtId="168" formatCode="0.0&quot;x&quot;"/>
+    <numFmt numFmtId="169" formatCode="0.0%"/>
+    <numFmt numFmtId="170" formatCode="#,##0\ &quot;€&quot;"/>
   </numFmts>
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -668,8 +891,80 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF666666"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF888888"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FFB45309"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -691,6 +986,21 @@
         <fgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0B1D3A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF1F5F9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -704,7 +1014,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -736,9 +1046,36 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="167" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="168" fontId="13" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="169" fontId="13" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="13" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="170" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="170" fontId="16" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="2" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="168" fontId="17" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="170" fontId="17" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="169" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="170" fontId="13" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="169" fontId="16" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -840,19 +1177,19 @@
                 <c:formatCode>"€"#,##0;\("€"#,##0\);\-</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>97115</c:v>
+                  <c:v>43820.35</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>533916.25</c:v>
+                  <c:v>299834.125</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1851023</c:v>
+                  <c:v>1093959.5</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4585217</c:v>
+                  <c:v>4204490.5</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8675782</c:v>
+                  <c:v>8019599</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -860,7 +1197,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-C27B-1A41-8454-F5C377455020}"/>
+              <c16:uniqueId val="{00000000-AD9B-C94E-A373-3EA19208852E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -916,19 +1253,19 @@
                 <c:formatCode>"€"#,##0;\("€"#,##0\);\-</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>594750.13500000001</c:v>
+                  <c:v>128848.845075</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>1283918.07125</c:v>
+                  <c:v>367448.98962499999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>2631840.8670000001</c:v>
+                  <c:v>1015570.8255</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>4258232.0930000003</c:v>
+                  <c:v>3515191.0245000003</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>5409396.4780000001</c:v>
+                  <c:v>3964367.1710000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -936,7 +1273,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-C27B-1A41-8454-F5C377455020}"/>
+              <c16:uniqueId val="{00000001-AD9B-C94E-A373-3EA19208852E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -992,19 +1329,19 @@
                 <c:formatCode>"€"#,##0;\("€"#,##0\);\-</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>-741398.4542588474</c:v>
+                  <c:v>-84535.543219165629</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-12813212.13124685</c:v>
+                  <c:v>736897.49902988155</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5564738.7851692578</c:v>
+                  <c:v>754189.75664060563</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>3769932.030225195</c:v>
+                  <c:v>1003170.7435800898</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>2935053.5681276959</c:v>
+                  <c:v>455146.92713259591</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1012,7 +1349,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-C27B-1A41-8454-F5C377455020}"/>
+              <c16:uniqueId val="{00000002-AD9B-C94E-A373-3EA19208852E}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1198,19 +1535,19 @@
                 <c:formatCode>"€"#,##0;\("€"#,##0\);\-</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>-497635.13500000001</c:v>
+                  <c:v>-85028.495075000013</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-750001.82125000004</c:v>
+                  <c:v>-67614.864624999987</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-780817.86700000009</c:v>
+                  <c:v>78388.674499999965</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>326984.90699999966</c:v>
+                  <c:v>689299.47549999971</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3266385.5219999999</c:v>
+                  <c:v>4055231.8289999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1218,7 +1555,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-53A7-244C-ADB0-D1C9E21EC42D}"/>
+              <c16:uniqueId val="{00000000-F947-8C4F-8769-AA0FD288EA19}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1274,19 +1611,19 @@
                 <c:formatCode>"€"#,##0;\("€"#,##0\);\-</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>-497635.13500000001</c:v>
+                  <c:v>-85028.495075000013</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-1247636.95625</c:v>
+                  <c:v>-152643.3597</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-2028454.8232500001</c:v>
+                  <c:v>-74254.685200000036</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-1701469.9162500005</c:v>
+                  <c:v>615044.79029999964</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1564915.6057499994</c:v>
+                  <c:v>4670276.6192999994</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1294,7 +1631,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-53A7-244C-ADB0-D1C9E21EC42D}"/>
+              <c16:uniqueId val="{00000001-F947-8C4F-8769-AA0FD288EA19}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1480,19 +1817,19 @@
                 <c:formatCode>"€"#,##0;\("€"#,##0\);\-</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>1252364.865</c:v>
+                  <c:v>1664971.504925</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>502363.04374999995</c:v>
+                  <c:v>1597356.6403000001</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>4721545.1767499996</c:v>
+                  <c:v>6675745.3147999998</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5048530.0837499993</c:v>
+                  <c:v>7365044.7902999995</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>8314915.6057499992</c:v>
+                  <c:v>11420276.6193</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1500,7 +1837,7 @@
           <c:smooth val="1"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-70B8-A64F-8AD4-FC1499F35BAB}"/>
+              <c16:uniqueId val="{00000000-665B-AB43-A85E-CAB97FF773E1}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1608,7 +1945,7 @@
   <c:date1904 val="0"/>
   <c:lang val="de-DE"/>
   <c:roundedCorners val="1"/>
-  <c:style val="11"/>
+  <c:style val="2"/>
   <c:chart>
     <c:title>
       <c:tx>
@@ -1685,26 +2022,26 @@
                 <c:formatCode>"€"#,##0;\("€"#,##0\);\-</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>440000</c:v>
+                  <c:v>56000</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>720000</c:v>
+                  <c:v>114000</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1170000</c:v>
+                  <c:v>174000</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1512000</c:v>
+                  <c:v>216000</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1670000</c:v>
+                  <c:v>244000</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-2632-EC42-9940-BE18F1EE268E}"/>
+              <c16:uniqueId val="{00000000-16D2-0041-A5BD-EAED40A17DA9}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1758,26 +2095,26 @@
                 <c:formatCode>"€"#,##0;\("€"#,##0\);\-</c:formatCode>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>154750.13500000001</c:v>
+                  <c:v>72848.845075000005</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>563918.07125000004</c:v>
+                  <c:v>253448.98962499999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1461840.8670000001</c:v>
+                  <c:v>841570.82550000004</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>2746232.0930000003</c:v>
+                  <c:v>3299191.0245000003</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>3739396.4780000001</c:v>
+                  <c:v>3720367.1710000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-2632-EC42-9940-BE18F1EE268E}"/>
+              <c16:uniqueId val="{00000001-16D2-0041-A5BD-EAED40A17DA9}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2304,255 +2641,255 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
+      <c r="A1" s="46" t="s">
+        <v>31</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="23" t="s">
-        <v>1</v>
-      </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
+      <c r="A3" s="48" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
-        <v>2</v>
+        <v>33</v>
       </c>
       <c r="B4" s="4">
         <v>500000</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>3</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
-        <v>4</v>
+        <v>35</v>
       </c>
       <c r="B5" s="4">
         <v>6000000</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>5</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="3" t="s">
-        <v>6</v>
+        <v>37</v>
       </c>
       <c r="B6" s="4">
-        <v>12000</v>
+        <v>2600</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>7</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="3" t="s">
-        <v>8</v>
+        <v>39</v>
       </c>
       <c r="B7" s="4">
-        <v>95000</v>
+        <v>5000</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>9</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>10</v>
+        <v>41</v>
       </c>
       <c r="B8" s="6">
         <v>1.2E-2</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>11</v>
+        <v>42</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="23" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
+      <c r="A10" s="48" t="s">
+        <v>43</v>
+      </c>
+      <c r="B10" s="47"/>
+      <c r="C10" s="47"/>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
-        <v>13</v>
+        <v>44</v>
       </c>
       <c r="B11" s="6">
         <v>0.04</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>14</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="3" t="s">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="B12" s="6">
         <v>0.01</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="B13" s="6">
         <v>0.03</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="B14" s="6">
         <v>0.02</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="23" t="s">
-        <v>21</v>
-      </c>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
+      <c r="A16" s="48" t="s">
+        <v>52</v>
+      </c>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="3" t="s">
-        <v>22</v>
+        <v>53</v>
       </c>
       <c r="B17" s="7">
         <v>4</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="3" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="B18" s="7">
         <v>18</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>25</v>
+        <v>56</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>26</v>
+        <v>57</v>
       </c>
       <c r="B19" s="7">
         <v>240</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>27</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A21" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
+      <c r="A21" s="48" t="s">
+        <v>59</v>
+      </c>
+      <c r="B21" s="47"/>
+      <c r="C21" s="47"/>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
-        <v>29</v>
+        <v>60</v>
       </c>
       <c r="B22" s="7">
         <v>0.12</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="B23" s="7">
         <v>0.18</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>32</v>
+        <v>63</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
-        <v>33</v>
+        <v>64</v>
       </c>
       <c r="B24" s="6">
         <v>0.3</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>34</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="3" t="s">
-        <v>35</v>
+        <v>66</v>
       </c>
       <c r="B25" s="6">
         <v>0.15</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>36</v>
+        <v>67</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="3" t="s">
-        <v>37</v>
+        <v>68</v>
       </c>
       <c r="B26" s="6">
         <v>2.9000000000000001E-2</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="3" t="s">
-        <v>39</v>
+        <v>70</v>
       </c>
       <c r="B27" s="6">
         <v>0.1</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>40</v>
+        <v>71</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="3" t="s">
-        <v>41</v>
+        <v>72</v>
       </c>
       <c r="B28" s="6">
         <v>0.05</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>42</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A30" s="26" t="s">
-        <v>43</v>
-      </c>
-      <c r="B30" s="24"/>
-      <c r="C30" s="24"/>
+      <c r="A30" s="49" t="s">
+        <v>74</v>
+      </c>
+      <c r="B30" s="47"/>
+      <c r="C30" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -2564,6 +2901,345 @@
     <mergeCell ref="A16:C16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:E31"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="40" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" ht="17" x14ac:dyDescent="0.2">
+      <c r="A1" s="24" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" s="29" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="34" t="s">
+        <v>240</v>
+      </c>
+      <c r="B4" s="40">
+        <v>1500000</v>
+      </c>
+      <c r="E4" s="29" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="42" t="s">
+        <v>242</v>
+      </c>
+      <c r="B6" s="42"/>
+      <c r="C6" s="42"/>
+      <c r="D6" s="42"/>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A7" s="37" t="s">
+        <v>243</v>
+      </c>
+      <c r="B7" s="39" t="s">
+        <v>244</v>
+      </c>
+      <c r="C7" s="39" t="s">
+        <v>245</v>
+      </c>
+      <c r="D7" s="39" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A8" s="30">
+        <v>0.05</v>
+      </c>
+      <c r="B8" s="33">
+        <f t="shared" ref="B8:B13" si="0">$B$4*A8/(1-A8)</f>
+        <v>78947.368421052641</v>
+      </c>
+      <c r="C8" s="33">
+        <f t="shared" ref="C8:C13" si="1">$B$4+B8</f>
+        <v>1578947.3684210526</v>
+      </c>
+      <c r="D8" s="43">
+        <f t="shared" ref="D8:D13" si="2">1-A8</f>
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A9" s="30">
+        <v>0.1</v>
+      </c>
+      <c r="B9" s="33">
+        <f t="shared" si="0"/>
+        <v>166666.66666666666</v>
+      </c>
+      <c r="C9" s="33">
+        <f t="shared" si="1"/>
+        <v>1666666.6666666667</v>
+      </c>
+      <c r="D9" s="43">
+        <f t="shared" si="2"/>
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A10" s="30">
+        <v>0.15</v>
+      </c>
+      <c r="B10" s="33">
+        <f t="shared" si="0"/>
+        <v>264705.8823529412</v>
+      </c>
+      <c r="C10" s="33">
+        <f t="shared" si="1"/>
+        <v>1764705.8823529412</v>
+      </c>
+      <c r="D10" s="43">
+        <f t="shared" si="2"/>
+        <v>0.85</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A11" s="30">
+        <v>0.2</v>
+      </c>
+      <c r="B11" s="33">
+        <f t="shared" si="0"/>
+        <v>375000</v>
+      </c>
+      <c r="C11" s="33">
+        <f t="shared" si="1"/>
+        <v>1875000</v>
+      </c>
+      <c r="D11" s="43">
+        <f t="shared" si="2"/>
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A12" s="30">
+        <v>0.25</v>
+      </c>
+      <c r="B12" s="33">
+        <f t="shared" si="0"/>
+        <v>500000</v>
+      </c>
+      <c r="C12" s="33">
+        <f t="shared" si="1"/>
+        <v>2000000</v>
+      </c>
+      <c r="D12" s="43">
+        <f t="shared" si="2"/>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="30">
+        <v>0.3</v>
+      </c>
+      <c r="B13" s="33">
+        <f t="shared" si="0"/>
+        <v>642857.14285714284</v>
+      </c>
+      <c r="C13" s="33">
+        <f t="shared" si="1"/>
+        <v>2142857.1428571427</v>
+      </c>
+      <c r="D13" s="43">
+        <f t="shared" si="2"/>
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="42" t="s">
+        <v>247</v>
+      </c>
+      <c r="B15" s="42"/>
+      <c r="C15" s="42"/>
+      <c r="D15" s="42"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="37" t="s">
+        <v>244</v>
+      </c>
+      <c r="B16" s="39" t="s">
+        <v>248</v>
+      </c>
+      <c r="C16" s="39" t="s">
+        <v>245</v>
+      </c>
+      <c r="D16" s="39" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="44">
+        <v>100000</v>
+      </c>
+      <c r="B17" s="43">
+        <f t="shared" ref="B17:B22" si="3">A17/($B$4+A17)</f>
+        <v>6.25E-2</v>
+      </c>
+      <c r="C17" s="33">
+        <f t="shared" ref="C17:C22" si="4">$B$4+A17</f>
+        <v>1600000</v>
+      </c>
+      <c r="D17" s="43">
+        <f t="shared" ref="D17:D22" si="5">$B$4/($B$4+A17)</f>
+        <v>0.9375</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="44">
+        <v>250000</v>
+      </c>
+      <c r="B18" s="43">
+        <f t="shared" si="3"/>
+        <v>0.14285714285714285</v>
+      </c>
+      <c r="C18" s="33">
+        <f t="shared" si="4"/>
+        <v>1750000</v>
+      </c>
+      <c r="D18" s="43">
+        <f t="shared" si="5"/>
+        <v>0.8571428571428571</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="44">
+        <v>500000</v>
+      </c>
+      <c r="B19" s="43">
+        <f t="shared" si="3"/>
+        <v>0.25</v>
+      </c>
+      <c r="C19" s="33">
+        <f t="shared" si="4"/>
+        <v>2000000</v>
+      </c>
+      <c r="D19" s="43">
+        <f t="shared" si="5"/>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="44">
+        <v>750000</v>
+      </c>
+      <c r="B20" s="43">
+        <f t="shared" si="3"/>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="C20" s="33">
+        <f t="shared" si="4"/>
+        <v>2250000</v>
+      </c>
+      <c r="D20" s="43">
+        <f t="shared" si="5"/>
+        <v>0.66666666666666663</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="44">
+        <v>1000000</v>
+      </c>
+      <c r="B21" s="43">
+        <f t="shared" si="3"/>
+        <v>0.4</v>
+      </c>
+      <c r="C21" s="33">
+        <f t="shared" si="4"/>
+        <v>2500000</v>
+      </c>
+      <c r="D21" s="43">
+        <f t="shared" si="5"/>
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="44">
+        <v>1500000</v>
+      </c>
+      <c r="B22" s="43">
+        <f t="shared" si="3"/>
+        <v>0.5</v>
+      </c>
+      <c r="C22" s="33">
+        <f t="shared" si="4"/>
+        <v>3000000</v>
+      </c>
+      <c r="D22" s="43">
+        <f t="shared" si="5"/>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="42" t="s">
+        <v>249</v>
+      </c>
+      <c r="B24" s="42"/>
+      <c r="C24" s="42"/>
+      <c r="D24" s="42"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="27" t="s">
+        <v>250</v>
+      </c>
+      <c r="B25" s="32">
+        <f>'3_Investment'!C20</f>
+        <v>1500000</v>
+      </c>
+      <c r="E25" s="29" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="34" t="s">
+        <v>252</v>
+      </c>
+      <c r="B26" s="45">
+        <f>B25/($B$4+B25)</f>
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="27" t="s">
+        <v>253</v>
+      </c>
+      <c r="B27" s="33">
+        <f>$B$4+B25</f>
+        <v>3000000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="41" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A30" s="41" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A31" s="41" t="s">
+        <v>256</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -2579,48 +3255,48 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
-        <v>44</v>
-      </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
+      <c r="A1" s="46" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
+      <c r="A3" s="48" t="s">
+        <v>1</v>
+      </c>
+      <c r="B3" s="47"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="47"/>
+      <c r="E3" s="47"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>46</v>
+        <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>47</v>
+        <v>3</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>50</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B5" s="7">
+        <v>7</v>
+      </c>
+      <c r="B5" s="23">
         <v>0</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="23">
         <v>0</v>
       </c>
       <c r="D5" s="8">
@@ -2628,17 +3304,17 @@
         <v>0</v>
       </c>
       <c r="E5" t="s">
-        <v>52</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B6" s="7">
+        <v>9</v>
+      </c>
+      <c r="B6" s="23">
         <v>4.99</v>
       </c>
-      <c r="C6" s="7">
+      <c r="C6" s="23">
         <v>49</v>
       </c>
       <c r="D6" s="8">
@@ -2646,17 +3322,17 @@
         <v>4.6273333333333335</v>
       </c>
       <c r="E6" t="s">
-        <v>54</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>55</v>
-      </c>
-      <c r="B7" s="7">
+        <v>11</v>
+      </c>
+      <c r="B7" s="23">
         <v>9.99</v>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="23">
         <v>99</v>
       </c>
       <c r="D7" s="8">
@@ -2664,38 +3340,38 @@
         <v>9.2940000000000005</v>
       </c>
       <c r="E7" t="s">
-        <v>56</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="B9" s="24"/>
-      <c r="C9" s="24"/>
-      <c r="D9" s="24"/>
-      <c r="E9" s="24"/>
+      <c r="A9" s="48" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="47"/>
+      <c r="C9" s="47"/>
+      <c r="D9" s="47"/>
+      <c r="E9" s="47"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
-        <v>46</v>
+        <v>2</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>47</v>
+        <v>3</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>48</v>
+        <v>4</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>58</v>
+        <v>14</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>59</v>
+        <v>15</v>
       </c>
       <c r="B11" s="7">
         <v>0</v>
@@ -2708,30 +3384,30 @@
         <v>0</v>
       </c>
       <c r="E11" t="s">
-        <v>60</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="B12" s="7">
-        <v>29</v>
+        <v>0</v>
       </c>
       <c r="C12" s="7">
-        <v>290</v>
+        <v>0</v>
       </c>
       <c r="D12" s="8">
         <f>B12*0.5+(C12/12)*0.5</f>
-        <v>26.583333333333336</v>
+        <v>0</v>
       </c>
       <c r="E12" t="s">
-        <v>62</v>
+        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="B13" s="7">
         <v>79</v>
@@ -2744,12 +3420,12 @@
         <v>72.416666666666657</v>
       </c>
       <c r="E13" t="s">
-        <v>64</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="B14" s="7">
         <v>199</v>
@@ -2762,21 +3438,21 @@
         <v>182.41666666666669</v>
       </c>
       <c r="E14" t="s">
-        <v>66</v>
+        <v>22</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="23" t="s">
-        <v>67</v>
-      </c>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
+      <c r="A17" s="48" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" s="47"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="47"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>68</v>
+        <v>24</v>
       </c>
       <c r="B18" s="6">
         <v>0.8</v>
@@ -2784,7 +3460,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>69</v>
+        <v>25</v>
       </c>
       <c r="B19" s="6">
         <v>0.2</v>
@@ -2792,7 +3468,7 @@
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>70</v>
+        <v>26</v>
       </c>
       <c r="B20" s="6">
         <v>0.55000000000000004</v>
@@ -2800,7 +3476,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="B21" s="6">
         <v>0.35</v>
@@ -2808,7 +3484,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>28</v>
       </c>
       <c r="B22" s="6">
         <v>0.1</v>
@@ -2816,7 +3492,7 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A24" s="9" t="s">
-        <v>73</v>
+        <v>29</v>
       </c>
       <c r="B24" s="10">
         <f>D6*B18+D7*B19</f>
@@ -2825,11 +3501,11 @@
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A25" s="9" t="s">
-        <v>74</v>
+        <v>30</v>
       </c>
       <c r="B25" s="10">
         <f>D12*B20+D13*B21+D14*B22</f>
-        <v>58.208333333333329</v>
+        <v>43.587499999999999</v>
       </c>
     </row>
   </sheetData>
@@ -2840,6 +3516,7 @@
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -2853,14 +3530,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="46" t="s">
         <v>75</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
@@ -2882,7 +3559,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="12" t="s">
         <v>82</v>
       </c>
@@ -2907,10 +3584,10 @@
         <v>88</v>
       </c>
       <c r="B5" s="7">
-        <v>220000</v>
+        <v>0</v>
       </c>
       <c r="C5" s="7">
-        <v>320000</v>
+        <v>0</v>
       </c>
       <c r="D5" s="7">
         <v>380000</v>
@@ -2927,10 +3604,10 @@
         <v>89</v>
       </c>
       <c r="B6" s="7">
-        <v>45000</v>
+        <v>0</v>
       </c>
       <c r="C6" s="7">
-        <v>60000</v>
+        <v>0</v>
       </c>
       <c r="D6" s="7">
         <v>70000</v>
@@ -2967,10 +3644,10 @@
         <v>91</v>
       </c>
       <c r="B8" s="7">
-        <v>60000</v>
+        <v>10000</v>
       </c>
       <c r="C8" s="7">
-        <v>180000</v>
+        <v>30000</v>
       </c>
       <c r="D8" s="7">
         <v>350000</v>
@@ -3088,11 +3765,11 @@
       </c>
       <c r="B14" s="14">
         <f>SUM(B5:B13)</f>
-        <v>467500</v>
+        <v>152500</v>
       </c>
       <c r="C14" s="14">
         <f>SUM(C5:C13)</f>
-        <v>858000</v>
+        <v>328000</v>
       </c>
       <c r="D14" s="14">
         <f>SUM(D5:D13)</f>
@@ -3113,32 +3790,32 @@
       </c>
       <c r="B15" s="14">
         <f>B14</f>
-        <v>467500</v>
+        <v>152500</v>
       </c>
       <c r="C15" s="14">
         <f>B15+C14</f>
-        <v>1325500</v>
+        <v>480500</v>
       </c>
       <c r="D15" s="14">
         <f>C15+D14</f>
-        <v>2634500</v>
+        <v>1789500</v>
       </c>
       <c r="E15" s="14">
         <f>D15+E14</f>
-        <v>4205300</v>
+        <v>3360300</v>
       </c>
       <c r="F15" s="14">
         <f>E15+F14</f>
-        <v>5673800</v>
+        <v>4828800</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="25" t="s">
+      <c r="A17" s="46" t="s">
         <v>99</v>
       </c>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
+      <c r="B17" s="47"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
@@ -3199,29 +3876,30 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:H26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="44" customWidth="1"/>
     <col min="2" max="7" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A1" s="46" t="s">
         <v>110</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
         <v>111</v>
       </c>
@@ -3241,97 +3919,102 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="23" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A4" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>113</v>
       </c>
       <c r="B5" s="7">
-        <v>220000</v>
+        <v>0</v>
       </c>
       <c r="C5" s="7">
-        <v>320000</v>
+        <v>0</v>
       </c>
       <c r="D5" s="7">
-        <v>480000</v>
+        <v>0</v>
       </c>
       <c r="E5" s="7">
-        <v>600000</v>
+        <v>0</v>
       </c>
       <c r="F5" s="7">
-        <v>660000</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>114</v>
       </c>
       <c r="B6" s="7">
-        <v>60000</v>
+        <v>0</v>
       </c>
       <c r="C6" s="7">
-        <v>140000</v>
+        <v>0</v>
       </c>
       <c r="D6" s="7">
-        <v>260000</v>
+        <v>0</v>
       </c>
       <c r="E6" s="7">
-        <v>360000</v>
+        <v>0</v>
       </c>
       <c r="F6" s="7">
-        <v>380000</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>115</v>
       </c>
       <c r="B7" s="7">
-        <v>30000</v>
+        <v>0</v>
       </c>
       <c r="C7" s="7">
-        <v>80000</v>
+        <v>0</v>
       </c>
       <c r="D7" s="7">
-        <v>160000</v>
+        <v>0</v>
       </c>
       <c r="E7" s="7">
-        <v>220000</v>
+        <v>0</v>
       </c>
       <c r="F7" s="7">
-        <v>260000</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>116</v>
       </c>
       <c r="B8" s="7">
-        <v>80000</v>
+        <f>2000*6</f>
+        <v>12000</v>
       </c>
       <c r="C8" s="7">
-        <v>90000</v>
+        <f>2000*12</f>
+        <v>24000</v>
       </c>
       <c r="D8" s="7">
-        <v>120000</v>
+        <f t="shared" ref="D8:E8" si="0">2000*12</f>
+        <v>24000</v>
       </c>
       <c r="E8" s="7">
-        <v>140000</v>
+        <f t="shared" si="0"/>
+        <v>24000</v>
       </c>
       <c r="F8" s="7">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+        <f>2000*12</f>
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>117</v>
       </c>
@@ -3351,12 +4034,12 @@
         <v>42000</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>118</v>
       </c>
       <c r="B10" s="7">
-        <v>8000</v>
+        <v>2000</v>
       </c>
       <c r="C10" s="7">
         <v>14000</v>
@@ -3371,7 +4054,7 @@
         <v>36000</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>119</v>
       </c>
@@ -3390,8 +4073,12 @@
       <c r="F11" s="7">
         <v>36000</v>
       </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="H11" s="7">
+        <f>12*20+18*12+25*12</f>
+        <v>756</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>120</v>
       </c>
@@ -3411,7 +4098,7 @@
         <v>16000</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>121</v>
       </c>
@@ -3431,40 +4118,40 @@
         <v>90000</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A14" s="2" t="s">
         <v>122</v>
       </c>
       <c r="B14" s="14">
         <f>SUM(B5:B13)</f>
-        <v>440000</v>
+        <v>56000</v>
       </c>
       <c r="C14" s="14">
         <f>SUM(C5:C13)</f>
-        <v>720000</v>
+        <v>114000</v>
       </c>
       <c r="D14" s="14">
         <f>SUM(D5:D13)</f>
-        <v>1170000</v>
+        <v>174000</v>
       </c>
       <c r="E14" s="14">
         <f>SUM(E5:E13)</f>
-        <v>1512000</v>
+        <v>216000</v>
       </c>
       <c r="F14" s="14">
         <f>SUM(F5:F13)</f>
-        <v>1670000</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="23" t="s">
+        <v>244000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="A16" s="48" t="s">
         <v>123</v>
       </c>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="47"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
@@ -3472,15 +4159,15 @@
       </c>
       <c r="B17" s="16">
         <f>'5_Umsatz_Prognose'!B26</f>
-        <v>21600</v>
+        <v>10800</v>
       </c>
       <c r="C17" s="16">
         <f>'5_Umsatz_Prognose'!C26</f>
-        <v>108000</v>
+        <v>43200</v>
       </c>
       <c r="D17" s="16">
         <f>'5_Umsatz_Prognose'!D26</f>
-        <v>316800</v>
+        <v>144000</v>
       </c>
       <c r="E17" s="16">
         <f>'5_Umsatz_Prognose'!E26</f>
@@ -3497,15 +4184,15 @@
       </c>
       <c r="B18" s="16">
         <f>'5_Umsatz_Prognose'!B27</f>
-        <v>1620</v>
+        <v>810</v>
       </c>
       <c r="C18" s="16">
         <f>'5_Umsatz_Prognose'!C27</f>
-        <v>8100</v>
+        <v>3240</v>
       </c>
       <c r="D18" s="16">
         <f>'5_Umsatz_Prognose'!D27</f>
-        <v>23760</v>
+        <v>10800</v>
       </c>
       <c r="E18" s="16">
         <f>'5_Umsatz_Prognose'!E27</f>
@@ -3522,15 +4209,15 @@
       </c>
       <c r="B19" s="16">
         <f>'5_Umsatz_Prognose'!B28</f>
-        <v>15013.8</v>
+        <v>3753.45</v>
       </c>
       <c r="C19" s="16">
         <f>'5_Umsatz_Prognose'!C28</f>
-        <v>37534.5</v>
+        <v>15013.8</v>
       </c>
       <c r="D19" s="16">
         <f>'5_Umsatz_Prognose'!D28</f>
-        <v>110101.2</v>
+        <v>50046</v>
       </c>
       <c r="E19" s="16">
         <f>'5_Umsatz_Prognose'!E28</f>
@@ -3547,23 +4234,23 @@
       </c>
       <c r="B20" s="16">
         <f>'5_Umsatz_Prognose'!B29</f>
-        <v>2816.335</v>
+        <v>635.39507500000002</v>
       </c>
       <c r="C20" s="16">
         <f>'5_Umsatz_Prognose'!C29</f>
-        <v>15483.571250000001</v>
+        <v>8695.1896250000009</v>
       </c>
       <c r="D20" s="16">
         <f>'5_Umsatz_Prognose'!D29</f>
-        <v>53679.667000000001</v>
+        <v>31724.825500000003</v>
       </c>
       <c r="E20" s="16">
         <f>'5_Umsatz_Prognose'!E29</f>
-        <v>132971.29300000001</v>
+        <v>121930.22450000001</v>
       </c>
       <c r="F20" s="16">
         <f>'5_Umsatz_Prognose'!F29</f>
-        <v>251597.67800000001</v>
+        <v>232568.37100000001</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -3572,19 +4259,19 @@
       </c>
       <c r="B21" s="16">
         <f>'5_Umsatz_Prognose'!B30</f>
-        <v>60000</v>
+        <v>30000</v>
       </c>
       <c r="C21" s="16">
         <f>'5_Umsatz_Prognose'!C30</f>
-        <v>240000</v>
+        <v>60000</v>
       </c>
       <c r="D21" s="16">
         <f>'5_Umsatz_Prognose'!D30</f>
-        <v>580000</v>
+        <v>280000</v>
       </c>
       <c r="E21" s="16">
         <f>'5_Umsatz_Prognose'!E30</f>
-        <v>1040000</v>
+        <v>1520000</v>
       </c>
       <c r="F21" s="16">
         <f>'5_Umsatz_Prognose'!F30</f>
@@ -3597,19 +4284,19 @@
       </c>
       <c r="B22" s="16">
         <f>'5_Umsatz_Prognose'!B31</f>
-        <v>10500</v>
+        <v>5250</v>
       </c>
       <c r="C22" s="16">
         <f>'5_Umsatz_Prognose'!C31</f>
-        <v>42000</v>
+        <v>10500</v>
       </c>
       <c r="D22" s="16">
         <f>'5_Umsatz_Prognose'!D31</f>
-        <v>101500</v>
+        <v>49000</v>
       </c>
       <c r="E22" s="16">
         <f>'5_Umsatz_Prognose'!E31</f>
-        <v>182000</v>
+        <v>266000</v>
       </c>
       <c r="F22" s="16">
         <f>'5_Umsatz_Prognose'!F31</f>
@@ -3622,7 +4309,7 @@
       </c>
       <c r="B23" s="16">
         <f>'5_Umsatz_Prognose'!B32</f>
-        <v>43200</v>
+        <v>21600</v>
       </c>
       <c r="C23" s="16">
         <f>'5_Umsatz_Prognose'!C32</f>
@@ -3647,23 +4334,23 @@
       </c>
       <c r="B24" s="14">
         <f>SUM(B17:B23)</f>
-        <v>154750.13500000001</v>
+        <v>72848.845075000005</v>
       </c>
       <c r="C24" s="14">
         <f>SUM(C17:C23)</f>
-        <v>563918.07125000004</v>
+        <v>253448.98962499999</v>
       </c>
       <c r="D24" s="14">
         <f>SUM(D17:D23)</f>
-        <v>1461840.8670000001</v>
+        <v>841570.82550000004</v>
       </c>
       <c r="E24" s="14">
         <f>SUM(E17:E23)</f>
-        <v>2746232.0930000003</v>
+        <v>3299191.0245000003</v>
       </c>
       <c r="F24" s="14">
         <f>SUM(F17:F23)</f>
-        <v>3739396.4780000001</v>
+        <v>3720367.1710000001</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
@@ -3672,23 +4359,23 @@
       </c>
       <c r="B26" s="17">
         <f>B14+B24</f>
-        <v>594750.13500000001</v>
+        <v>128848.845075</v>
       </c>
       <c r="C26" s="17">
         <f>C14+C24</f>
-        <v>1283918.07125</v>
+        <v>367448.98962499999</v>
       </c>
       <c r="D26" s="17">
         <f>D14+D24</f>
-        <v>2631840.8670000001</v>
+        <v>1015570.8255</v>
       </c>
       <c r="E26" s="17">
         <f>E14+E24</f>
-        <v>4258232.0930000003</v>
+        <v>3515191.0245000003</v>
       </c>
       <c r="F26" s="17">
         <f>F14+F24</f>
-        <v>5409396.4780000001</v>
+        <v>3964367.1710000001</v>
       </c>
     </row>
   </sheetData>
@@ -3698,10 +4385,370 @@
     <mergeCell ref="A4:F4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9767F7A4-89EF-8648-9BC3-9EA62E5853BF}">
+  <dimension ref="A1:C33"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="44" customWidth="1"/>
+    <col min="2" max="4" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="46" t="s">
+        <v>257</v>
+      </c>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="48" t="s">
+        <v>135</v>
+      </c>
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>136</v>
+      </c>
+      <c r="B5" s="4">
+        <v>15000</v>
+      </c>
+      <c r="C5" s="4">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>137</v>
+      </c>
+      <c r="B6" s="18">
+        <f>'1_Annahmen'!B11</f>
+        <v>0.04</v>
+      </c>
+      <c r="C6" s="18">
+        <f>'1_Annahmen'!B11</f>
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>138</v>
+      </c>
+      <c r="B7" s="18">
+        <f>'1_Annahmen'!B12</f>
+        <v>0.01</v>
+      </c>
+      <c r="C7" s="18">
+        <f>'1_Annahmen'!B12</f>
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>139</v>
+      </c>
+      <c r="B8" s="19">
+        <f>B5*B6</f>
+        <v>600</v>
+      </c>
+      <c r="C8" s="19">
+        <f>C5*C6</f>
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>140</v>
+      </c>
+      <c r="B9" s="19">
+        <f>B5*B7</f>
+        <v>150</v>
+      </c>
+      <c r="C9" s="19">
+        <f>C5*C7</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="9" t="s">
+        <v>141</v>
+      </c>
+      <c r="B10" s="20">
+        <f>B8+B9</f>
+        <v>750</v>
+      </c>
+      <c r="C10" s="20">
+        <f>C8+C9</f>
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="48" t="s">
+        <v>142</v>
+      </c>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>143</v>
+      </c>
+      <c r="B13" s="4">
+        <v>180</v>
+      </c>
+      <c r="C13" s="4">
+        <v>650</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>144</v>
+      </c>
+      <c r="B14" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="C14" s="6">
+        <v>0.45</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="9" t="s">
+        <v>145</v>
+      </c>
+      <c r="B15" s="20">
+        <f>B13*B14</f>
+        <v>54</v>
+      </c>
+      <c r="C15" s="20">
+        <f>C13*C14</f>
+        <v>292.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="48" t="s">
+        <v>146</v>
+      </c>
+      <c r="B17" s="47"/>
+      <c r="C17" s="47"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>147</v>
+      </c>
+      <c r="B18" s="8">
+        <f>B10*'2_Pricing'!B24*12/2</f>
+        <v>25023</v>
+      </c>
+      <c r="C18" s="8">
+        <f>C10*'2_Pricing'!B24*12</f>
+        <v>100092</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>148</v>
+      </c>
+      <c r="B19" s="8">
+        <f>B15*'2_Pricing'!B25*12/2</f>
+        <v>14122.349999999999</v>
+      </c>
+      <c r="C19" s="8">
+        <f>C15*'2_Pricing'!B25*12</f>
+        <v>152992.125</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>149</v>
+      </c>
+      <c r="B20" s="8">
+        <f>B10*60*0.8*'1_Annahmen'!B27/2</f>
+        <v>1800</v>
+      </c>
+      <c r="C20" s="8">
+        <f>C10*80*1.5*'1_Annahmen'!B27</f>
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>150</v>
+      </c>
+      <c r="B21" s="8">
+        <f>B10*20*'1_Annahmen'!B28/2</f>
+        <v>375</v>
+      </c>
+      <c r="C21" s="8">
+        <f>C10*50*'1_Annahmen'!B28</f>
+        <v>3750</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>151</v>
+      </c>
+      <c r="B22" s="7">
+        <v>2500</v>
+      </c>
+      <c r="C22" s="7">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A23" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="B23" s="14">
+        <f>SUM(B18:B22)</f>
+        <v>43820.35</v>
+      </c>
+      <c r="C23" s="14">
+        <f>SUM(C18:C22)</f>
+        <v>299834.125</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="48" t="s">
+        <v>153</v>
+      </c>
+      <c r="B25" s="47"/>
+      <c r="C25" s="47"/>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>154</v>
+      </c>
+      <c r="B26" s="8">
+        <f>B5*'1_Annahmen'!B22*12/2</f>
+        <v>10800</v>
+      </c>
+      <c r="C26" s="8">
+        <f>C5*'1_Annahmen'!B22*12</f>
+        <v>43200</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>155</v>
+      </c>
+      <c r="B27" s="8">
+        <f>B10*'1_Annahmen'!B23*12/2</f>
+        <v>810</v>
+      </c>
+      <c r="C27" s="8">
+        <f>C10*'1_Annahmen'!B23*12</f>
+        <v>3240</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>156</v>
+      </c>
+      <c r="B28" s="8">
+        <f>B18*'1_Annahmen'!B24/2</f>
+        <v>3753.45</v>
+      </c>
+      <c r="C28" s="8">
+        <f>C18*'1_Annahmen'!B25</f>
+        <v>15013.8</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>157</v>
+      </c>
+      <c r="B29" s="8">
+        <f>B23*'1_Annahmen'!B26/2</f>
+        <v>635.39507500000002</v>
+      </c>
+      <c r="C29" s="8">
+        <f>C23*'1_Annahmen'!B26</f>
+        <v>8695.1896250000009</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>158</v>
+      </c>
+      <c r="B30" s="8">
+        <f>B5*'1_Annahmen'!B17/2</f>
+        <v>30000</v>
+      </c>
+      <c r="C30" s="8">
+        <f>MAX(0,C5-B5)*'1_Annahmen'!B17</f>
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>159</v>
+      </c>
+      <c r="B31" s="8">
+        <f>B10*('1_Annahmen'!B18-'1_Annahmen'!B17)/2</f>
+        <v>5250</v>
+      </c>
+      <c r="C31" s="8">
+        <f>MAX(0,C10-B10)*('1_Annahmen'!B18-'1_Annahmen'!B17)</f>
+        <v>10500</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>160</v>
+      </c>
+      <c r="B32" s="8">
+        <f>B13*'1_Annahmen'!B19/2</f>
+        <v>21600</v>
+      </c>
+      <c r="C32" s="8">
+        <f>MAX(0,C13-B13)*'1_Annahmen'!B19</f>
+        <v>112800</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="9" t="s">
+        <v>131</v>
+      </c>
+      <c r="B33" s="10">
+        <f>SUM(B26:B32)</f>
+        <v>72848.845075000005</v>
+      </c>
+      <c r="C33" s="10">
+        <f>SUM(C26:C32)</f>
+        <v>253448.98962499999</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A25:C25"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -3711,14 +4758,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="46" t="s">
         <v>133</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
@@ -3741,14 +4788,14 @@
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="48" t="s">
         <v>135</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
-      <c r="F4" s="24"/>
+      <c r="B4" s="47"/>
+      <c r="C4" s="47"/>
+      <c r="D4" s="47"/>
+      <c r="E4" s="47"/>
+      <c r="F4" s="47"/>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -3758,10 +4805,10 @@
         <v>15000</v>
       </c>
       <c r="C5" s="4">
-        <v>75000</v>
+        <v>30000</v>
       </c>
       <c r="D5" s="4">
-        <v>220000</v>
+        <v>100000</v>
       </c>
       <c r="E5" s="4">
         <v>480000</v>
@@ -3830,11 +4877,11 @@
       </c>
       <c r="C8" s="19">
         <f>C5*C6</f>
-        <v>3000</v>
+        <v>1200</v>
       </c>
       <c r="D8" s="19">
         <f>D5*D6</f>
-        <v>8800</v>
+        <v>4000</v>
       </c>
       <c r="E8" s="19">
         <f>E5*E6</f>
@@ -3855,11 +4902,11 @@
       </c>
       <c r="C9" s="19">
         <f>C5*C7</f>
-        <v>750</v>
+        <v>300</v>
       </c>
       <c r="D9" s="19">
         <f>D5*D7</f>
-        <v>2200</v>
+        <v>1000</v>
       </c>
       <c r="E9" s="19">
         <f>E5*E7</f>
@@ -3880,11 +4927,11 @@
       </c>
       <c r="C10" s="20">
         <f>C8+C9</f>
-        <v>3750</v>
+        <v>1500</v>
       </c>
       <c r="D10" s="20">
         <f>D8+D9</f>
-        <v>11000</v>
+        <v>5000</v>
       </c>
       <c r="E10" s="20">
         <f>E8+E9</f>
@@ -3896,14 +4943,14 @@
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="23" t="s">
+      <c r="A12" s="48" t="s">
         <v>142</v>
       </c>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="24"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47"/>
+      <c r="F12" s="47"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -3971,30 +5018,30 @@
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="48" t="s">
         <v>146</v>
       </c>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
+      <c r="B17" s="47"/>
+      <c r="C17" s="47"/>
+      <c r="D17" s="47"/>
+      <c r="E17" s="47"/>
+      <c r="F17" s="47"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>147</v>
       </c>
       <c r="B18" s="8">
-        <f>B10*'2_Pricing'!B24*12</f>
-        <v>50046</v>
+        <f>B10*'2_Pricing'!B24*12/2</f>
+        <v>25023</v>
       </c>
       <c r="C18" s="8">
         <f>C10*'2_Pricing'!B24*12</f>
-        <v>250230</v>
+        <v>100092</v>
       </c>
       <c r="D18" s="8">
         <f>D10*'2_Pricing'!B24*12</f>
-        <v>734008</v>
+        <v>333640</v>
       </c>
       <c r="E18" s="8">
         <f>E10*'2_Pricing'!B24*12</f>
@@ -4010,24 +5057,24 @@
         <v>148</v>
       </c>
       <c r="B19" s="8">
-        <f>B15*'2_Pricing'!B25*12</f>
-        <v>37718.999999999993</v>
+        <f>B15*'2_Pricing'!B25*12/2</f>
+        <v>14122.349999999999</v>
       </c>
       <c r="C19" s="8">
         <f>C15*'2_Pricing'!B25*12</f>
-        <v>204311.25</v>
+        <v>152992.125</v>
       </c>
       <c r="D19" s="8">
         <f>D15*'2_Pricing'!B25*12</f>
-        <v>691515</v>
+        <v>517819.5</v>
       </c>
       <c r="E19" s="8">
         <f>E15*'2_Pricing'!B25*12</f>
-        <v>1515745</v>
+        <v>1135018.5</v>
       </c>
       <c r="F19" s="8">
         <f>F15*'2_Pricing'!B25*12</f>
-        <v>2612390</v>
+        <v>1956207</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -4035,16 +5082,16 @@
         <v>149</v>
       </c>
       <c r="B20" s="8">
-        <f>B10*60*0.8*'1_Annahmen'!B27</f>
-        <v>3600</v>
+        <f>B10*60*0.8*'1_Annahmen'!B27/2</f>
+        <v>1800</v>
       </c>
       <c r="C20" s="8">
         <f>C10*80*1.5*'1_Annahmen'!B27</f>
-        <v>45000</v>
+        <v>18000</v>
       </c>
       <c r="D20" s="8">
         <f>D10*100*2.5*'1_Annahmen'!B27</f>
-        <v>275000</v>
+        <v>125000</v>
       </c>
       <c r="E20" s="8">
         <f>E10*120*3.5*'1_Annahmen'!B27</f>
@@ -4060,16 +5107,16 @@
         <v>150</v>
       </c>
       <c r="B21" s="8">
-        <f>B10*20*'1_Annahmen'!B28</f>
-        <v>750</v>
+        <f>B10*20*'1_Annahmen'!B28/2</f>
+        <v>375</v>
       </c>
       <c r="C21" s="8">
         <f>C10*50*'1_Annahmen'!B28</f>
-        <v>9375</v>
+        <v>3750</v>
       </c>
       <c r="D21" s="8">
         <f>D10*110*'1_Annahmen'!B28</f>
-        <v>60500</v>
+        <v>27500</v>
       </c>
       <c r="E21" s="8">
         <f>E10*200*'1_Annahmen'!B28</f>
@@ -4085,7 +5132,7 @@
         <v>151</v>
       </c>
       <c r="B22" s="7">
-        <v>5000</v>
+        <v>2500</v>
       </c>
       <c r="C22" s="7">
         <v>25000</v>
@@ -4106,50 +5153,50 @@
       </c>
       <c r="B23" s="14">
         <f>SUM(B18:B22)</f>
-        <v>97115</v>
+        <v>43820.35</v>
       </c>
       <c r="C23" s="14">
         <f>SUM(C18:C22)</f>
-        <v>533916.25</v>
+        <v>299834.125</v>
       </c>
       <c r="D23" s="14">
         <f>SUM(D18:D22)</f>
-        <v>1851023</v>
+        <v>1093959.5</v>
       </c>
       <c r="E23" s="14">
         <f>SUM(E18:E22)</f>
-        <v>4585217</v>
+        <v>4204490.5</v>
       </c>
       <c r="F23" s="14">
         <f>SUM(F18:F22)</f>
-        <v>8675782</v>
+        <v>8019599</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A25" s="23" t="s">
+      <c r="A25" s="48" t="s">
         <v>153</v>
       </c>
-      <c r="B25" s="24"/>
-      <c r="C25" s="24"/>
-      <c r="D25" s="24"/>
-      <c r="E25" s="24"/>
-      <c r="F25" s="24"/>
+      <c r="B25" s="47"/>
+      <c r="C25" s="47"/>
+      <c r="D25" s="47"/>
+      <c r="E25" s="47"/>
+      <c r="F25" s="47"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>154</v>
       </c>
       <c r="B26" s="8">
-        <f>B5*'1_Annahmen'!B22*12</f>
-        <v>21600</v>
+        <f>B5*'1_Annahmen'!B22*12/2</f>
+        <v>10800</v>
       </c>
       <c r="C26" s="8">
         <f>C5*'1_Annahmen'!B22*12</f>
-        <v>108000</v>
+        <v>43200</v>
       </c>
       <c r="D26" s="8">
         <f>D5*'1_Annahmen'!B22*12</f>
-        <v>316800</v>
+        <v>144000</v>
       </c>
       <c r="E26" s="8">
         <f>E5*'1_Annahmen'!B22*12</f>
@@ -4165,16 +5212,16 @@
         <v>155</v>
       </c>
       <c r="B27" s="8">
-        <f>B10*'1_Annahmen'!B23*12</f>
-        <v>1620</v>
+        <f>B10*'1_Annahmen'!B23*12/2</f>
+        <v>810</v>
       </c>
       <c r="C27" s="8">
         <f>C10*'1_Annahmen'!B23*12</f>
-        <v>8100</v>
+        <v>3240</v>
       </c>
       <c r="D27" s="8">
         <f>D10*'1_Annahmen'!B23*12</f>
-        <v>23760</v>
+        <v>10800</v>
       </c>
       <c r="E27" s="8">
         <f>E10*'1_Annahmen'!B23*12</f>
@@ -4190,16 +5237,16 @@
         <v>156</v>
       </c>
       <c r="B28" s="8">
-        <f>B18*'1_Annahmen'!B24</f>
-        <v>15013.8</v>
+        <f>B18*'1_Annahmen'!B24/2</f>
+        <v>3753.45</v>
       </c>
       <c r="C28" s="8">
         <f>C18*'1_Annahmen'!B25</f>
-        <v>37534.5</v>
+        <v>15013.8</v>
       </c>
       <c r="D28" s="8">
         <f>D18*'1_Annahmen'!B25</f>
-        <v>110101.2</v>
+        <v>50046</v>
       </c>
       <c r="E28" s="8">
         <f>E18*'1_Annahmen'!B25</f>
@@ -4215,24 +5262,24 @@
         <v>157</v>
       </c>
       <c r="B29" s="8">
-        <f>B23*'1_Annahmen'!B26</f>
-        <v>2816.335</v>
+        <f>B23*'1_Annahmen'!B26/2</f>
+        <v>635.39507500000002</v>
       </c>
       <c r="C29" s="8">
         <f>C23*'1_Annahmen'!B26</f>
-        <v>15483.571250000001</v>
+        <v>8695.1896250000009</v>
       </c>
       <c r="D29" s="8">
         <f>D23*'1_Annahmen'!B26</f>
-        <v>53679.667000000001</v>
+        <v>31724.825500000003</v>
       </c>
       <c r="E29" s="8">
         <f>E23*'1_Annahmen'!B26</f>
-        <v>132971.29300000001</v>
+        <v>121930.22450000001</v>
       </c>
       <c r="F29" s="8">
         <f>F23*'1_Annahmen'!B26</f>
-        <v>251597.67800000001</v>
+        <v>232568.37100000001</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
@@ -4240,20 +5287,20 @@
         <v>158</v>
       </c>
       <c r="B30" s="8">
-        <f>B5*'1_Annahmen'!B17</f>
-        <v>60000</v>
+        <f>B5*'1_Annahmen'!B17/2</f>
+        <v>30000</v>
       </c>
       <c r="C30" s="8">
         <f>MAX(0,C5-B5)*'1_Annahmen'!B17</f>
-        <v>240000</v>
+        <v>60000</v>
       </c>
       <c r="D30" s="8">
         <f>MAX(0,D5-C5)*'1_Annahmen'!B17</f>
-        <v>580000</v>
+        <v>280000</v>
       </c>
       <c r="E30" s="8">
         <f>MAX(0,E5-D5)*'1_Annahmen'!B17</f>
-        <v>1040000</v>
+        <v>1520000</v>
       </c>
       <c r="F30" s="8">
         <f>MAX(0,F5-E5)*'1_Annahmen'!B17</f>
@@ -4265,20 +5312,20 @@
         <v>159</v>
       </c>
       <c r="B31" s="8">
-        <f>B10*('1_Annahmen'!B18-'1_Annahmen'!B17)</f>
-        <v>10500</v>
+        <f>B10*('1_Annahmen'!B18-'1_Annahmen'!B17)/2</f>
+        <v>5250</v>
       </c>
       <c r="C31" s="8">
         <f>MAX(0,C10-B10)*('1_Annahmen'!B18-'1_Annahmen'!B17)</f>
-        <v>42000</v>
+        <v>10500</v>
       </c>
       <c r="D31" s="8">
         <f>MAX(0,D10-C10)*('1_Annahmen'!B18-'1_Annahmen'!B17)</f>
-        <v>101500</v>
+        <v>49000</v>
       </c>
       <c r="E31" s="8">
         <f>MAX(0,E10-D10)*('1_Annahmen'!B18-'1_Annahmen'!B17)</f>
-        <v>182000</v>
+        <v>266000</v>
       </c>
       <c r="F31" s="8">
         <f>MAX(0,F10-E10)*('1_Annahmen'!B18-'1_Annahmen'!B17)</f>
@@ -4290,8 +5337,8 @@
         <v>160</v>
       </c>
       <c r="B32" s="8">
-        <f>B13*'1_Annahmen'!B19</f>
-        <v>43200</v>
+        <f>B13*'1_Annahmen'!B19/2</f>
+        <v>21600</v>
       </c>
       <c r="C32" s="8">
         <f>MAX(0,C13-B13)*'1_Annahmen'!B19</f>
@@ -4316,23 +5363,23 @@
       </c>
       <c r="B33" s="10">
         <f>SUM(B26:B32)</f>
-        <v>154750.13500000001</v>
+        <v>72848.845075000005</v>
       </c>
       <c r="C33" s="10">
         <f>SUM(C26:C32)</f>
-        <v>563918.07125000004</v>
+        <v>253448.98962499999</v>
       </c>
       <c r="D33" s="10">
         <f>SUM(D26:D32)</f>
-        <v>1461840.8670000001</v>
+        <v>841570.82550000004</v>
       </c>
       <c r="E33" s="10">
         <f>SUM(E26:E32)</f>
-        <v>2746232.0930000003</v>
+        <v>3299191.0245000003</v>
       </c>
       <c r="F33" s="10">
         <f>SUM(F26:F32)</f>
-        <v>3739396.4780000001</v>
+        <v>3720367.1710000001</v>
       </c>
     </row>
   </sheetData>
@@ -4344,10 +5391,11 @@
     <mergeCell ref="A25:F25"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -4357,14 +5405,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="46" t="s">
         <v>161</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="2" t="s">
@@ -4392,23 +5440,23 @@
       </c>
       <c r="B4" s="16">
         <f>'5_Umsatz_Prognose'!B23</f>
-        <v>97115</v>
+        <v>43820.35</v>
       </c>
       <c r="C4" s="16">
         <f>'5_Umsatz_Prognose'!C23</f>
-        <v>533916.25</v>
+        <v>299834.125</v>
       </c>
       <c r="D4" s="16">
         <f>'5_Umsatz_Prognose'!D23</f>
-        <v>1851023</v>
+        <v>1093959.5</v>
       </c>
       <c r="E4" s="16">
         <f>'5_Umsatz_Prognose'!E23</f>
-        <v>4585217</v>
+        <v>4204490.5</v>
       </c>
       <c r="F4" s="16">
         <f>'5_Umsatz_Prognose'!F23</f>
-        <v>8675782</v>
+        <v>8019599</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -4417,23 +5465,23 @@
       </c>
       <c r="B5" s="16">
         <f>-'5_Umsatz_Prognose'!B33</f>
-        <v>-154750.13500000001</v>
+        <v>-72848.845075000005</v>
       </c>
       <c r="C5" s="16">
         <f>-'5_Umsatz_Prognose'!C33</f>
-        <v>-563918.07125000004</v>
+        <v>-253448.98962499999</v>
       </c>
       <c r="D5" s="16">
         <f>-'5_Umsatz_Prognose'!D33</f>
-        <v>-1461840.8670000001</v>
+        <v>-841570.82550000004</v>
       </c>
       <c r="E5" s="16">
         <f>-'5_Umsatz_Prognose'!E33</f>
-        <v>-2746232.0930000003</v>
+        <v>-3299191.0245000003</v>
       </c>
       <c r="F5" s="16">
         <f>-'5_Umsatz_Prognose'!F33</f>
-        <v>-3739396.4780000001</v>
+        <v>-3720367.1710000001</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -4442,23 +5490,23 @@
       </c>
       <c r="B6" s="10">
         <f>B4+B5</f>
-        <v>-57635.135000000009</v>
+        <v>-29028.495075000006</v>
       </c>
       <c r="C6" s="10">
         <f>C4+C5</f>
-        <v>-30001.821250000037</v>
+        <v>46385.135375000013</v>
       </c>
       <c r="D6" s="10">
         <f>D4+D5</f>
-        <v>389182.13299999991</v>
+        <v>252388.67449999996</v>
       </c>
       <c r="E6" s="10">
         <f>E4+E5</f>
-        <v>1838984.9069999997</v>
+        <v>905299.47549999971</v>
       </c>
       <c r="F6" s="10">
         <f>F4+F5</f>
-        <v>4936385.5219999999</v>
+        <v>4299231.8289999999</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -4467,23 +5515,23 @@
       </c>
       <c r="B7" s="21">
         <f>IFERROR(B6/B4,0)</f>
-        <v>-0.59347304741800966</v>
+        <v>-0.66244325011096461</v>
       </c>
       <c r="C7" s="21">
         <f>IFERROR(C6/C4,0)</f>
-        <v>-5.619199874512161E-2</v>
+        <v>0.15470265559332186</v>
       </c>
       <c r="D7" s="21">
         <f>IFERROR(D6/D4,0)</f>
-        <v>0.21025245661453149</v>
+        <v>0.23071116846647427</v>
       </c>
       <c r="E7" s="21">
         <f>IFERROR(E6/E4,0)</f>
-        <v>0.40106823886415838</v>
+        <v>0.21531728410374568</v>
       </c>
       <c r="F7" s="21">
         <f>IFERROR(F6/F4,0)</f>
-        <v>0.56898450445158721</v>
+        <v>0.53609062360848714</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -4492,23 +5540,23 @@
       </c>
       <c r="B8" s="16">
         <f>-'4_Kosten'!B14</f>
-        <v>-440000</v>
+        <v>-56000</v>
       </c>
       <c r="C8" s="16">
         <f>-'4_Kosten'!C14</f>
-        <v>-720000</v>
+        <v>-114000</v>
       </c>
       <c r="D8" s="16">
         <f>-'4_Kosten'!D14</f>
-        <v>-1170000</v>
+        <v>-174000</v>
       </c>
       <c r="E8" s="16">
         <f>-'4_Kosten'!E14</f>
-        <v>-1512000</v>
+        <v>-216000</v>
       </c>
       <c r="F8" s="16">
         <f>-'4_Kosten'!F14</f>
-        <v>-1670000</v>
+        <v>-244000</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -4517,23 +5565,23 @@
       </c>
       <c r="B9" s="14">
         <f>B6+B8</f>
-        <v>-497635.13500000001</v>
+        <v>-85028.495075000013</v>
       </c>
       <c r="C9" s="14">
         <f>C6+C8</f>
-        <v>-750001.82125000004</v>
+        <v>-67614.864624999987</v>
       </c>
       <c r="D9" s="14">
         <f>D6+D8</f>
-        <v>-780817.86700000009</v>
+        <v>78388.674499999965</v>
       </c>
       <c r="E9" s="14">
         <f>E6+E8</f>
-        <v>326984.90699999966</v>
+        <v>689299.47549999971</v>
       </c>
       <c r="F9" s="14">
         <f>F6+F8</f>
-        <v>3266385.5219999999</v>
+        <v>4055231.8289999999</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -4542,34 +5590,34 @@
       </c>
       <c r="B10" s="21">
         <f>IFERROR(B9/B4,0)</f>
-        <v>-5.1241840601348914</v>
+        <v>-1.9403883144475116</v>
       </c>
       <c r="C10" s="21">
         <f>IFERROR(C9/C4,0)</f>
-        <v>-1.4047181018558623</v>
+        <v>-0.22550756897667998</v>
       </c>
       <c r="D10" s="21">
         <f>IFERROR(D9/D4,0)</f>
-        <v>-0.42183045105328248</v>
+        <v>7.1655920077479979E-2</v>
       </c>
       <c r="E10" s="21">
         <f>IFERROR(E9/E4,0)</f>
-        <v>7.1312853241187857E-2</v>
+        <v>0.1639436396633551</v>
       </c>
       <c r="F10" s="21">
         <f>IFERROR(F9/F4,0)</f>
-        <v>0.37649465166367713</v>
+        <v>0.50566516218579005</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" s="23" t="s">
+      <c r="A12" s="48" t="s">
         <v>169</v>
       </c>
-      <c r="B12" s="24"/>
-      <c r="C12" s="24"/>
-      <c r="D12" s="24"/>
-      <c r="E12" s="24"/>
-      <c r="F12" s="24"/>
+      <c r="B12" s="47"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47"/>
+      <c r="F12" s="47"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="9" t="s">
@@ -4577,23 +5625,23 @@
       </c>
       <c r="B13" s="10">
         <f>B9</f>
-        <v>-497635.13500000001</v>
+        <v>-85028.495075000013</v>
       </c>
       <c r="C13" s="10">
         <f>B13+C9</f>
-        <v>-1247636.95625</v>
+        <v>-152643.3597</v>
       </c>
       <c r="D13" s="10">
         <f>C13+D9</f>
-        <v>-2028454.8232500001</v>
+        <v>-74254.685200000036</v>
       </c>
       <c r="E13" s="10">
         <f>D13+E9</f>
-        <v>-1701469.9162500005</v>
+        <v>615044.79029999964</v>
       </c>
       <c r="F13" s="10">
         <f>E13+F9</f>
-        <v>1564915.6057499994</v>
+        <v>4670276.6192999994</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
@@ -4647,34 +5695,34 @@
       </c>
       <c r="B16" s="10">
         <f>B15+B13</f>
-        <v>1252364.865</v>
+        <v>1664971.504925</v>
       </c>
       <c r="C16" s="10">
         <f>C15+C13</f>
-        <v>502363.04374999995</v>
+        <v>1597356.6403000001</v>
       </c>
       <c r="D16" s="10">
         <f>D15+D13</f>
-        <v>4721545.1767499996</v>
+        <v>6675745.3147999998</v>
       </c>
       <c r="E16" s="10">
         <f>E15+E13</f>
-        <v>5048530.0837499993</v>
+        <v>7365044.7902999995</v>
       </c>
       <c r="F16" s="10">
         <f>F15+F13</f>
-        <v>8314915.6057499992</v>
+        <v>11420276.6193</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="23" t="s">
+      <c r="A18" s="48" t="s">
         <v>174</v>
       </c>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
+      <c r="B18" s="47"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="47"/>
+      <c r="E18" s="47"/>
+      <c r="F18" s="47"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="9" t="s">
@@ -4682,23 +5730,23 @@
       </c>
       <c r="B19" s="10">
         <f>IFERROR(-B8/IFERROR(B6/B4,0),0)</f>
-        <v>-741398.4542588474</v>
+        <v>-84535.543219165629</v>
       </c>
       <c r="C19" s="10">
         <f>IFERROR(-C8/IFERROR(C6/C4,0),0)</f>
-        <v>-12813212.13124685</v>
+        <v>736897.49902988155</v>
       </c>
       <c r="D19" s="10">
         <f>IFERROR(-D8/IFERROR(D6/D4,0),0)</f>
-        <v>5564738.7851692578</v>
+        <v>754189.75664060563</v>
       </c>
       <c r="E19" s="10">
         <f>IFERROR(-E8/IFERROR(E6/E4,0),0)</f>
-        <v>3769932.030225195</v>
+        <v>1003170.7435800898</v>
       </c>
       <c r="F19" s="10">
         <f>IFERROR(-F8/IFERROR(F6/F4,0),0)</f>
-        <v>2935053.5681276959</v>
+        <v>455146.92713259591</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
@@ -4707,23 +5755,23 @@
       </c>
       <c r="B20" s="16">
         <f>B4</f>
-        <v>97115</v>
+        <v>43820.35</v>
       </c>
       <c r="C20" s="16">
         <f>C4</f>
-        <v>533916.25</v>
+        <v>299834.125</v>
       </c>
       <c r="D20" s="16">
         <f>D4</f>
-        <v>1851023</v>
+        <v>1093959.5</v>
       </c>
       <c r="E20" s="16">
         <f>E4</f>
-        <v>4585217</v>
+        <v>4204490.5</v>
       </c>
       <c r="F20" s="16">
         <f>F4</f>
-        <v>8675782</v>
+        <v>8019599</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
@@ -4732,23 +5780,23 @@
       </c>
       <c r="B21" s="10">
         <f>B4-B19</f>
-        <v>838513.4542588474</v>
+        <v>128355.89321916562</v>
       </c>
       <c r="C21" s="10">
         <f>C4-C19</f>
-        <v>13347128.38124685</v>
+        <v>-437063.37402988155</v>
       </c>
       <c r="D21" s="10">
         <f>D4-D19</f>
-        <v>-3713715.7851692578</v>
+        <v>339769.74335939437</v>
       </c>
       <c r="E21" s="10">
         <f>E4-E19</f>
-        <v>815284.96977480501</v>
+        <v>3201319.7564199101</v>
       </c>
       <c r="F21" s="10">
         <f>F4-F19</f>
-        <v>5740728.4318723045</v>
+        <v>7564452.0728674037</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
@@ -4767,10 +5815,11 @@
     <mergeCell ref="A18:F18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
@@ -4780,14 +5829,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="25" t="s">
+      <c r="A1" s="46" t="s">
         <v>179</v>
       </c>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="24"/>
-      <c r="E1" s="24"/>
-      <c r="F1" s="24"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="9" t="s">
@@ -4815,23 +5864,23 @@
       </c>
       <c r="B4" s="16">
         <f>'6_GuV_Breakeven'!B4</f>
-        <v>97115</v>
+        <v>43820.35</v>
       </c>
       <c r="C4" s="16">
         <f>'6_GuV_Breakeven'!C4</f>
-        <v>533916.25</v>
+        <v>299834.125</v>
       </c>
       <c r="D4" s="16">
         <f>'6_GuV_Breakeven'!D4</f>
-        <v>1851023</v>
+        <v>1093959.5</v>
       </c>
       <c r="E4" s="16">
         <f>'6_GuV_Breakeven'!E4</f>
-        <v>4585217</v>
+        <v>4204490.5</v>
       </c>
       <c r="F4" s="16">
         <f>'6_GuV_Breakeven'!F4</f>
-        <v>8675782</v>
+        <v>8019599</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -4840,23 +5889,23 @@
       </c>
       <c r="B5" s="16">
         <f>'4_Kosten'!B14</f>
-        <v>440000</v>
+        <v>56000</v>
       </c>
       <c r="C5" s="16">
         <f>'4_Kosten'!C14</f>
-        <v>720000</v>
+        <v>114000</v>
       </c>
       <c r="D5" s="16">
         <f>'4_Kosten'!D14</f>
-        <v>1170000</v>
+        <v>174000</v>
       </c>
       <c r="E5" s="16">
         <f>'4_Kosten'!E14</f>
-        <v>1512000</v>
+        <v>216000</v>
       </c>
       <c r="F5" s="16">
         <f>'4_Kosten'!F14</f>
-        <v>1670000</v>
+        <v>244000</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -4865,23 +5914,23 @@
       </c>
       <c r="B6" s="16">
         <f>'5_Umsatz_Prognose'!B33</f>
-        <v>154750.13500000001</v>
+        <v>72848.845075000005</v>
       </c>
       <c r="C6" s="16">
         <f>'5_Umsatz_Prognose'!C33</f>
-        <v>563918.07125000004</v>
+        <v>253448.98962499999</v>
       </c>
       <c r="D6" s="16">
         <f>'5_Umsatz_Prognose'!D33</f>
-        <v>1461840.8670000001</v>
+        <v>841570.82550000004</v>
       </c>
       <c r="E6" s="16">
         <f>'5_Umsatz_Prognose'!E33</f>
-        <v>2746232.0930000003</v>
+        <v>3299191.0245000003</v>
       </c>
       <c r="F6" s="16">
         <f>'5_Umsatz_Prognose'!F33</f>
-        <v>3739396.4780000001</v>
+        <v>3720367.1710000001</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
@@ -4890,23 +5939,23 @@
       </c>
       <c r="B7" s="16">
         <f>'4_Kosten'!B26</f>
-        <v>594750.13500000001</v>
+        <v>128848.845075</v>
       </c>
       <c r="C7" s="16">
         <f>'4_Kosten'!C26</f>
-        <v>1283918.07125</v>
+        <v>367448.98962499999</v>
       </c>
       <c r="D7" s="16">
         <f>'4_Kosten'!D26</f>
-        <v>2631840.8670000001</v>
+        <v>1015570.8255</v>
       </c>
       <c r="E7" s="16">
         <f>'4_Kosten'!E26</f>
-        <v>4258232.0930000003</v>
+        <v>3515191.0245000003</v>
       </c>
       <c r="F7" s="16">
         <f>'4_Kosten'!F26</f>
-        <v>5409396.4780000001</v>
+        <v>3964367.1710000001</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -4915,23 +5964,23 @@
       </c>
       <c r="B8" s="16">
         <f>'6_GuV_Breakeven'!B9</f>
-        <v>-497635.13500000001</v>
+        <v>-85028.495075000013</v>
       </c>
       <c r="C8" s="16">
         <f>'6_GuV_Breakeven'!C9</f>
-        <v>-750001.82125000004</v>
+        <v>-67614.864624999987</v>
       </c>
       <c r="D8" s="16">
         <f>'6_GuV_Breakeven'!D9</f>
-        <v>-780817.86700000009</v>
+        <v>78388.674499999965</v>
       </c>
       <c r="E8" s="16">
         <f>'6_GuV_Breakeven'!E9</f>
-        <v>326984.90699999966</v>
+        <v>689299.47549999971</v>
       </c>
       <c r="F8" s="16">
         <f>'6_GuV_Breakeven'!F9</f>
-        <v>3266385.5219999999</v>
+        <v>4055231.8289999999</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
@@ -4940,23 +5989,23 @@
       </c>
       <c r="B9" s="16">
         <f>'6_GuV_Breakeven'!B13</f>
-        <v>-497635.13500000001</v>
+        <v>-85028.495075000013</v>
       </c>
       <c r="C9" s="16">
         <f>'6_GuV_Breakeven'!C13</f>
-        <v>-1247636.95625</v>
+        <v>-152643.3597</v>
       </c>
       <c r="D9" s="16">
         <f>'6_GuV_Breakeven'!D13</f>
-        <v>-2028454.8232500001</v>
+        <v>-74254.685200000036</v>
       </c>
       <c r="E9" s="16">
         <f>'6_GuV_Breakeven'!E13</f>
-        <v>-1701469.9162500005</v>
+        <v>615044.79029999964</v>
       </c>
       <c r="F9" s="16">
         <f>'6_GuV_Breakeven'!F13</f>
-        <v>1564915.6057499994</v>
+        <v>4670276.6192999994</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -4965,23 +6014,23 @@
       </c>
       <c r="B10" s="16">
         <f>'6_GuV_Breakeven'!B16</f>
-        <v>1252364.865</v>
+        <v>1664971.504925</v>
       </c>
       <c r="C10" s="16">
         <f>'6_GuV_Breakeven'!C16</f>
-        <v>502363.04374999995</v>
+        <v>1597356.6403000001</v>
       </c>
       <c r="D10" s="16">
         <f>'6_GuV_Breakeven'!D16</f>
-        <v>4721545.1767499996</v>
+        <v>6675745.3147999998</v>
       </c>
       <c r="E10" s="16">
         <f>'6_GuV_Breakeven'!E16</f>
-        <v>5048530.0837499993</v>
+        <v>7365044.7902999995</v>
       </c>
       <c r="F10" s="16">
         <f>'6_GuV_Breakeven'!F16</f>
-        <v>8314915.6057499992</v>
+        <v>11420276.6193</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -4990,23 +6039,23 @@
       </c>
       <c r="B11" s="16">
         <f>'6_GuV_Breakeven'!B19</f>
-        <v>-741398.4542588474</v>
+        <v>-84535.543219165629</v>
       </c>
       <c r="C11" s="16">
         <f>'6_GuV_Breakeven'!C19</f>
-        <v>-12813212.13124685</v>
+        <v>736897.49902988155</v>
       </c>
       <c r="D11" s="16">
         <f>'6_GuV_Breakeven'!D19</f>
-        <v>5564738.7851692578</v>
+        <v>754189.75664060563</v>
       </c>
       <c r="E11" s="16">
         <f>'6_GuV_Breakeven'!E19</f>
-        <v>3769932.030225195</v>
+        <v>1003170.7435800898</v>
       </c>
       <c r="F11" s="16">
         <f>'6_GuV_Breakeven'!F19</f>
-        <v>2935053.5681276959</v>
+        <v>455146.92713259591</v>
       </c>
     </row>
   </sheetData>
@@ -5014,6 +6063,468 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
+  <dimension ref="A1:G50"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="46" customWidth="1"/>
+    <col min="2" max="6" width="15" customWidth="1"/>
+    <col min="7" max="7" width="44" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="17" x14ac:dyDescent="0.2">
+      <c r="A1" s="24" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="25" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="26" t="s">
+        <v>188</v>
+      </c>
+      <c r="B4" s="26"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="27" t="s">
+        <v>189</v>
+      </c>
+      <c r="B5" s="28">
+        <v>4</v>
+      </c>
+      <c r="G5" s="29" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="27" t="s">
+        <v>191</v>
+      </c>
+      <c r="B6" s="28">
+        <v>12</v>
+      </c>
+      <c r="G6" s="29" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="27" t="s">
+        <v>193</v>
+      </c>
+      <c r="B7" s="30">
+        <v>0.5</v>
+      </c>
+      <c r="G7" s="29" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="27" t="s">
+        <v>195</v>
+      </c>
+      <c r="B8" s="30">
+        <v>0.5</v>
+      </c>
+      <c r="G8" s="29" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="27" t="s">
+        <v>197</v>
+      </c>
+      <c r="B9" s="31">
+        <v>5</v>
+      </c>
+      <c r="G9" s="29" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="27" t="s">
+        <v>199</v>
+      </c>
+      <c r="B10" s="30">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="G10" s="29" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="26" t="s">
+        <v>201</v>
+      </c>
+      <c r="B12" s="26"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="27" t="s">
+        <v>202</v>
+      </c>
+      <c r="B13" s="32">
+        <f>'5_Umsatz_Prognose'!F23</f>
+        <v>8019599</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="27" t="s">
+        <v>203</v>
+      </c>
+      <c r="B14" s="32">
+        <f>'6_GuV_Breakeven'!F9</f>
+        <v>4055231.8289999999</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="26" t="s">
+        <v>204</v>
+      </c>
+      <c r="B16" s="26"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="27" t="s">
+        <v>205</v>
+      </c>
+      <c r="B17" s="33">
+        <f>B13*B5</f>
+        <v>32078396</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" s="27" t="s">
+        <v>206</v>
+      </c>
+      <c r="B18" s="33">
+        <f>B14*B6</f>
+        <v>48662781.947999999</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" s="34" t="s">
+        <v>207</v>
+      </c>
+      <c r="B19" s="35">
+        <f>B7*B17+(1-B7)*B18</f>
+        <v>40370588.973999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" s="26" t="s">
+        <v>208</v>
+      </c>
+      <c r="B21" s="26"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="27" t="s">
+        <v>209</v>
+      </c>
+      <c r="B22" s="36">
+        <f>(1+B8)^B9</f>
+        <v>7.59375</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" s="34" t="s">
+        <v>210</v>
+      </c>
+      <c r="B23" s="35">
+        <f>B19/B22</f>
+        <v>5316291.5521316873</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="B24" s="33">
+        <f>B23*(1-B10)</f>
+        <v>2392331.1984592592</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" s="26" t="s">
+        <v>212</v>
+      </c>
+      <c r="B26" s="26"/>
+      <c r="C26" s="26"/>
+      <c r="D26" s="26"/>
+      <c r="E26" s="26"/>
+      <c r="F26" s="26"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A27" s="37" t="s">
+        <v>213</v>
+      </c>
+      <c r="B27" s="38">
+        <v>3</v>
+      </c>
+      <c r="C27" s="38">
+        <v>4</v>
+      </c>
+      <c r="D27" s="38">
+        <v>5</v>
+      </c>
+      <c r="E27" s="38">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" s="30">
+        <v>0.45</v>
+      </c>
+      <c r="B28" s="33">
+        <f t="shared" ref="B28:E31" si="0">($B$13*B$27)/(1+$A28)^$B$9</f>
+        <v>3753478.1888620676</v>
+      </c>
+      <c r="C28" s="33">
+        <f t="shared" si="0"/>
+        <v>5004637.5851494232</v>
+      </c>
+      <c r="D28" s="33">
+        <f t="shared" si="0"/>
+        <v>6255796.9814367797</v>
+      </c>
+      <c r="E28" s="33">
+        <f t="shared" si="0"/>
+        <v>7506956.3777241353</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" s="30">
+        <v>0.5</v>
+      </c>
+      <c r="B29" s="33">
+        <f t="shared" si="0"/>
+        <v>3168236.6419753088</v>
+      </c>
+      <c r="C29" s="33">
+        <f t="shared" si="0"/>
+        <v>4224315.5226337444</v>
+      </c>
+      <c r="D29" s="33">
+        <f t="shared" si="0"/>
+        <v>5280394.403292181</v>
+      </c>
+      <c r="E29" s="33">
+        <f t="shared" si="0"/>
+        <v>6336473.2839506175</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A30" s="30">
+        <v>0.55000000000000004</v>
+      </c>
+      <c r="B30" s="33">
+        <f t="shared" si="0"/>
+        <v>2689152.4097239203</v>
+      </c>
+      <c r="C30" s="33">
+        <f t="shared" si="0"/>
+        <v>3585536.5462985602</v>
+      </c>
+      <c r="D30" s="33">
+        <f t="shared" si="0"/>
+        <v>4481920.6828732006</v>
+      </c>
+      <c r="E30" s="33">
+        <f t="shared" si="0"/>
+        <v>5378304.8194478406</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A31" s="30">
+        <v>0.6</v>
+      </c>
+      <c r="B31" s="33">
+        <f t="shared" si="0"/>
+        <v>2294425.6782531724</v>
+      </c>
+      <c r="C31" s="33">
+        <f t="shared" si="0"/>
+        <v>3059234.2376708966</v>
+      </c>
+      <c r="D31" s="33">
+        <f t="shared" si="0"/>
+        <v>3824042.7970886207</v>
+      </c>
+      <c r="E31" s="33">
+        <f t="shared" si="0"/>
+        <v>4588851.3565063449</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A34" s="26" t="s">
+        <v>214</v>
+      </c>
+      <c r="B34" s="26"/>
+      <c r="C34" s="26"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A35" s="37" t="s">
+        <v>215</v>
+      </c>
+      <c r="B35" s="39" t="s">
+        <v>216</v>
+      </c>
+      <c r="C35" s="39" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A36" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="B36" s="33">
+        <v>175000</v>
+      </c>
+      <c r="C36" s="33">
+        <v>350000</v>
+      </c>
+      <c r="G36" s="29" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A37" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="B37" s="33">
+        <v>1300000</v>
+      </c>
+      <c r="C37" s="33">
+        <v>1700000</v>
+      </c>
+      <c r="G37" s="29" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A38" s="27" t="s">
+        <v>222</v>
+      </c>
+      <c r="B38" s="33">
+        <v>800000</v>
+      </c>
+      <c r="C38" s="33">
+        <v>1500000</v>
+      </c>
+      <c r="G38" s="29" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A39" s="27" t="s">
+        <v>224</v>
+      </c>
+      <c r="B39" s="33">
+        <f>B23*0.8</f>
+        <v>4253033.2417053496</v>
+      </c>
+      <c r="C39" s="33">
+        <f>B23*1.2</f>
+        <v>6379549.8625580249</v>
+      </c>
+      <c r="G39" s="29" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A40" s="37" t="s">
+        <v>226</v>
+      </c>
+      <c r="B40" s="40">
+        <v>1200000</v>
+      </c>
+      <c r="C40" s="40">
+        <v>1800000</v>
+      </c>
+      <c r="G40" s="29" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A42" s="26" t="s">
+        <v>228</v>
+      </c>
+      <c r="B42" s="26"/>
+      <c r="C42" s="26"/>
+    </row>
+    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A43" s="37" t="s">
+        <v>229</v>
+      </c>
+      <c r="B43" s="39" t="s">
+        <v>230</v>
+      </c>
+      <c r="C43" s="39" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A44" s="27" t="s">
+        <v>232</v>
+      </c>
+      <c r="B44" s="33">
+        <v>1200000</v>
+      </c>
+      <c r="C44" s="33">
+        <v>1800000</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A45" s="27" t="s">
+        <v>233</v>
+      </c>
+      <c r="B45" s="33">
+        <v>3000000</v>
+      </c>
+      <c r="C45" s="33">
+        <v>5000000</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A46" s="27" t="s">
+        <v>234</v>
+      </c>
+      <c r="B46" s="33">
+        <v>12000000</v>
+      </c>
+      <c r="C46" s="33">
+        <v>20000000</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A47" s="27" t="s">
+        <v>235</v>
+      </c>
+      <c r="B47" s="33">
+        <v>35000000</v>
+      </c>
+      <c r="C47" s="33">
+        <v>52000000</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A49" s="41" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A50" s="41" t="s">
+        <v>237</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
 </file>
</xml_diff>